<commit_message>
Update reports, scripts, and tests
</commit_message>
<xml_diff>
--- a/ipp_phase_breakdown_2026-02-27.xlsx
+++ b/ipp_phase_breakdown_2026-02-27.xlsx
@@ -6446,7 +6446,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-02-27 07:59:49 UTC</t>
+          <t>2026-02-27 11:19:17 UTC</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-02-27 07:59:49 UTC</t>
+          <t>2026-02-27 11:19:17 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>